<commit_message>
Regenerasi rata-rata 260622 dengan sheet Rp/km per bulan
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hasil_scraping/260622-Rata-rata Harga per Bulan.xlsx
+++ b/hasil_scraping/260622-Rata-rata Harga per Bulan.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Pivot Bulan x Rute" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Detail per Bulan-Rute" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Jumlah Data per Bulan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Rp per km per Bulan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10248,4 +10249,685 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>bulan</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>rata_rata_rp_per_km</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>jumlah_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1145</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2022-09</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C3" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1083</v>
+      </c>
+      <c r="C4" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1043</v>
+      </c>
+      <c r="C5" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2022-12</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1094</v>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>946</v>
+      </c>
+      <c r="C7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>829</v>
+      </c>
+      <c r="C8" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>871</v>
+      </c>
+      <c r="C9" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C10" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>810</v>
+      </c>
+      <c r="C11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>832</v>
+      </c>
+      <c r="C12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>890</v>
+      </c>
+      <c r="C13" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>921</v>
+      </c>
+      <c r="C14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>938</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1319</v>
+      </c>
+      <c r="C16" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1567</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2533</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1443</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2930</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1438</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3542</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1439</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4437</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1570</v>
+      </c>
+      <c r="C22" t="n">
+        <v>3219</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1484</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3927</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1597</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3025</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1563</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3165</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1601</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3269</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1707</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1620</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1659</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1638</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2527</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1717</v>
+      </c>
+      <c r="C30" t="n">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1685</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1827</v>
+      </c>
+      <c r="C32" t="n">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1798</v>
+      </c>
+      <c r="C33" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1682</v>
+      </c>
+      <c r="C34" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C35" t="n">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1412</v>
+      </c>
+      <c r="C36" t="n">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1392</v>
+      </c>
+      <c r="C37" t="n">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1353</v>
+      </c>
+      <c r="C38" t="n">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1383</v>
+      </c>
+      <c r="C39" t="n">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C40" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1109</v>
+      </c>
+      <c r="C41" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1304</v>
+      </c>
+      <c r="C42" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1178</v>
+      </c>
+      <c r="C43" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1254</v>
+      </c>
+      <c r="C44" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1306</v>
+      </c>
+      <c r="C45" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1346</v>
+      </c>
+      <c r="C46" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1836</v>
+      </c>
+      <c r="C47" t="n">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2097</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2291</v>
+      </c>
+      <c r="C49" t="n">
+        <v>5758</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2291</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3789</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2267</v>
+      </c>
+      <c r="C51" t="n">
+        <v>976</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>